<commit_message>
updating distance graph data
</commit_message>
<xml_diff>
--- a/tensile_burst_index.xlsx
+++ b/tensile_burst_index.xlsx
@@ -8,14 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/mjl9889_ads_northwestern_edu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{0BA2C7EC-AF05-EB44-BD45-8B30115AFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="14_{0BA2C7EC-AF05-EB44-BD45-8B30115AFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A639A3D-BB46-9E45-AD0B-A4DAA029ADE7}"/>
   <bookViews>
-    <workbookView xWindow="15100" yWindow="1660" windowWidth="13620" windowHeight="16200" xr2:uid="{322F6E6C-CBEF-ED47-ABD1-97FB92E66F46}"/>
+    <workbookView xWindow="11660" yWindow="1640" windowWidth="15420" windowHeight="16200" activeTab="1" xr2:uid="{322F6E6C-CBEF-ED47-ABD1-97FB92E66F46}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$B$2:$B$7</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$C$2:$C$7</definedName>
+    <definedName name="_xlchart.v2.5" hidden="1">Sheet2!$B$2:$B$7</definedName>
+    <definedName name="_xlchart.v2.6" hidden="1">Sheet2!$C$2:$C$7</definedName>
+    <definedName name="_xlchart.v5.0" hidden="1">Sheet2!$B$1</definedName>
+    <definedName name="_xlchart.v5.1" hidden="1">Sheet2!$B$2:$B$7</definedName>
+    <definedName name="_xlchart.v5.2" hidden="1">Sheet2!$C$2:$C$7</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -108,8 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -125,6 +135,1091 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-8B62-2C45-9DE6-083D16245EC9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Sheet2!$D$2:$D$7</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="6"/>
+                  <c:pt idx="0">
+                    <c:v>3.6422558638537881</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>3.6323845856100889</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>5.4502656408248207</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>4.3756814072528085</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5.1017766513244993</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>2.0512391918599393</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Sheet2!$D$2:$D$7</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="6"/>
+                  <c:pt idx="0">
+                    <c:v>3.6422558638537881</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>3.6323845856100889</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>5.4502656408248207</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>4.3756814072528085</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5.1017766513244993</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>2.0512391918599393</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>H1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>H2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>H3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>H4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>H5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>H6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>33.395000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>43.188000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>33.037999999999997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34.900999999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>42.096666666666664</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>43.543999999999997</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8B62-2C45-9DE6-083D16245EC9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="2131555456"/>
+        <c:axId val="2131556800"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="2131555456"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2131556800"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2131556800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Tensile</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Index</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2131555456"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>215900</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>660400</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{574DBD94-1C22-128D-BE29-C6DF97AF5C8F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1136,40 +2231,77 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C78BAF-05EF-984B-8770-296D3AC0C072}">
-  <dimension ref="B2:B7"/>
+  <dimension ref="B2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C2" s="1">
+        <v>33.395000000000003</v>
+      </c>
+      <c r="D2" s="1">
+        <v>3.6422558638537881</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C3" s="1">
+        <v>43.188000000000002</v>
+      </c>
+      <c r="D3" s="1">
+        <v>3.6323845856100889</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C4" s="1">
+        <v>33.037999999999997</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5.4502656408248207</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C5" s="1">
+        <v>34.900999999999996</v>
+      </c>
+      <c r="D5" s="1">
+        <v>4.3756814072528085</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C6" s="1">
+        <v>42.096666666666664</v>
+      </c>
+      <c r="D6" s="1">
+        <v>5.1017766513244993</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>9</v>
       </c>
+      <c r="C7" s="1">
+        <v>43.543999999999997</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2.0512391918599393</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
working on filtering out ASA and AKD data
</commit_message>
<xml_diff>
--- a/tensile_burst_index.xlsx
+++ b/tensile_burst_index.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/mjl9889_ads_northwestern_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/graphene-oxide-paper-coatings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="14_{0BA2C7EC-AF05-EB44-BD45-8B30115AFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A639A3D-BB46-9E45-AD0B-A4DAA029ADE7}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="14_{0BA2C7EC-AF05-EB44-BD45-8B30115AFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52DAB812-1CB6-264C-AE76-AFAA042086FC}"/>
   <bookViews>
     <workbookView xWindow="11660" yWindow="1640" windowWidth="15420" windowHeight="16200" activeTab="1" xr2:uid="{322F6E6C-CBEF-ED47-ABD1-97FB92E66F46}"/>
   </bookViews>
@@ -17,13 +17,13 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$B$2:$B$7</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$C$2:$C$7</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet2!$B$2:$B$7</definedName>
-    <definedName name="_xlchart.v2.6" hidden="1">Sheet2!$C$2:$C$7</definedName>
-    <definedName name="_xlchart.v5.0" hidden="1">Sheet2!$B$1</definedName>
-    <definedName name="_xlchart.v5.1" hidden="1">Sheet2!$B$2:$B$7</definedName>
-    <definedName name="_xlchart.v5.2" hidden="1">Sheet2!$C$2:$C$7</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$F$2:$F$7</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet2!$G$2:$G$7</definedName>
+    <definedName name="_xlchart.v2.0" hidden="1">Sheet2!$F$2:$F$7</definedName>
+    <definedName name="_xlchart.v2.1" hidden="1">Sheet2!$G$2:$G$7</definedName>
+    <definedName name="_xlchart.v5.2" hidden="1">Sheet2!$F$1</definedName>
+    <definedName name="_xlchart.v5.3" hidden="1">Sheet2!$F$2:$F$7</definedName>
+    <definedName name="_xlchart.v5.4" hidden="1">Sheet2!$G$2:$G$7</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="10">
   <si>
     <t>Condition</t>
   </si>
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -96,13 +96,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF83CBEB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC1E5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -117,9 +134,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -638,7 +661,548 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-A502-874D-B228-277403270328}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Sheet2!$H$2:$H$7</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="6"/>
+                  <c:pt idx="0">
+                    <c:v>2.68</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>1.84</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>2.96</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>1.34</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5.88</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>4.68</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Sheet2!$H$2:$H$7</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="6"/>
+                  <c:pt idx="0">
+                    <c:v>2.68</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>1.84</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>2.96</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>1.34</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>5.88</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>4.68</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$F$2:$F$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>H1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>H2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>H3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>H4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>H5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>H6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$G$2:$G$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>37.409999999999997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>38.75</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>39.11</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34.49</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>43.54</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>47.69</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A502-874D-B228-277403270328}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="29820223"/>
+        <c:axId val="29822463"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="29820223"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="29822463"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="29822463"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="50"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Tensile</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Index</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="29820223"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1181,6 +1745,509 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1214,6 +2281,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>469900</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9399890-AD28-27E1-502A-C47F57F3773D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2231,10 +3334,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C78BAF-05EF-984B-8770-296D3AC0C072}">
-  <dimension ref="B2:D7"/>
+  <dimension ref="B2:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -2244,8 +3347,17 @@
       <c r="D2" s="1">
         <v>3.6422558638537881</v>
       </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1">
+        <v>37.409999999999997</v>
+      </c>
+      <c r="H2" s="1">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>5</v>
       </c>
@@ -2255,8 +3367,17 @@
       <c r="D3" s="1">
         <v>3.6323845856100889</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="1">
+        <v>38.75</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -2266,8 +3387,17 @@
       <c r="D4" s="1">
         <v>5.4502656408248207</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="1">
+        <v>39.11</v>
+      </c>
+      <c r="H4" s="1">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -2277,8 +3407,17 @@
       <c r="D5" s="1">
         <v>4.3756814072528085</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1">
+        <v>34.49</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>8</v>
       </c>
@@ -2288,8 +3427,17 @@
       <c r="D6" s="1">
         <v>5.1017766513244993</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="1">
+        <v>43.54</v>
+      </c>
+      <c r="H6" s="1">
+        <v>5.88</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>9</v>
       </c>
@@ -2299,6 +3447,33 @@
       <c r="D7" s="1">
         <v>2.0512391918599393</v>
       </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="1">
+        <v>47.69</v>
+      </c>
+      <c r="H7" s="1">
+        <v>4.68</v>
+      </c>
+    </row>
+    <row r="20" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="11:11" ht="24" x14ac:dyDescent="0.2">
+      <c r="K25" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
working on data cleaning for the honors thesis section
</commit_message>
<xml_diff>
--- a/tensile_burst_index.xlsx
+++ b/tensile_burst_index.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -16,18 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$J$2:$J$7</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$K$2:$K$7</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet2!$J$2:$J$7</definedName>
-    <definedName name="_xlchart.v2.6" hidden="1">Sheet2!$K$2:$K$7</definedName>
-    <definedName name="_xlchart.v5.0" hidden="1">Sheet2!$J$1</definedName>
-    <definedName name="_xlchart.v5.1" hidden="1">Sheet2!$J$2:$J$7</definedName>
-    <definedName name="_xlchart.v5.2" hidden="1">Sheet2!$K$2:$K$7</definedName>
-    <definedName name="_xlchart.v5.7" hidden="1">Sheet2!$F$1</definedName>
-    <definedName name="_xlchart.v5.8" hidden="1">Sheet2!$F$2:$F$7</definedName>
-    <definedName name="_xlchart.v5.9" hidden="1">Sheet2!$G$2:$G$7</definedName>
-  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">

</xml_diff>